<commit_message>
Update and add Excel data files
Updated several existing Excel files in the data directory and added a new file, FIFA Days.xlsx. These changes likely reflect updated datasets for competitions, stadiums, teams, and scheduling.
</commit_message>
<xml_diff>
--- a/data/CAF CC.xlsx
+++ b/data/CAF CC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Computer Science\Graduation Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibram\OneDrive\Documents\GitHub\Egyptian-Premier-League-Schedule-Optimizer\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51059D25-A827-4D0F-8C15-19C22BFE05F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D831C0B-F518-41AA-8A32-F2FB5B775937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="18">
   <si>
     <t>Round Name</t>
   </si>
@@ -130,41 +130,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -200,6 +176,29 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -228,8 +227,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2D979AB1-B7F5-4073-9EE2-DBB4A6781A59}" name="CAF_CC" displayName="CAF_CC" ref="A1:B25" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:B25" xr:uid="{2D979AB1-B7F5-4073-9EE2-DBB4A6781A59}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{55EB70C4-BD9D-4E1D-9155-7BF8FB823987}" uniqueName="1" name="Round Name" queryTableFieldId="1" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{8C20053E-E872-4BE2-BFF5-909B291D846F}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{55EB70C4-BD9D-4E1D-9155-7BF8FB823987}" uniqueName="1" name="Round Name" queryTableFieldId="1" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{8C20053E-E872-4BE2-BFF5-909B291D846F}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -239,8 +238,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42B61CA6-C148-4432-97ED-F9CFAF80C10F}" name="Table1" displayName="Table1" ref="A1:B25" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:B25" xr:uid="{42B61CA6-C148-4432-97ED-F9CFAF80C10F}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{099424EA-71A1-427F-8375-A212B96B7E76}" name="Round Name" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{F05D1CF4-DEC8-4BAF-B818-52097C7BC73B}" name="Date" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{099424EA-71A1-427F-8375-A212B96B7E76}" name="Round Name" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{F05D1CF4-DEC8-4BAF-B818-52097C7BC73B}" name="Date" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -460,178 +459,194 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
         <v>46250</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
         <v>46251</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
         <v>46252</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <v>46257</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="5">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4">
         <v>46258</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4">
         <v>46259</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>46278</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4">
         <v>46279</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="5">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="4">
         <v>46280</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>46285</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="4">
         <v>46286</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="5">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="4">
         <v>46287</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="4">
         <v>46353</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="4">
         <v>46364</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="4">
         <v>46371</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="4">
         <v>46392</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="4">
         <v>46399</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="4">
         <v>46406</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="4">
         <v>46479</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="4">
         <v>46486</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="A22" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22" s="4">
         <v>46497</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="5">
+      <c r="B23" s="4">
         <v>46504</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="A24" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24" s="4">
         <v>46524</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25" s="4">
         <v>46532</v>
       </c>
     </row>

</xml_diff>